<commit_message>
daily: 收银合规看板 2026-08-10 更新
</commit_message>
<xml_diff>
--- a/cashier/不合规明细_20260810.xlsx
+++ b/cashier/不合规明细_20260810.xlsx
@@ -476,27 +476,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海中庚漫游城授权体验店</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海中庚漫游城授权体验店</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>LSD2026080800943589</t>
+          <t>LSD2026080100898820</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -516,7 +516,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>150****1153</t>
+          <t>150****6552</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -533,27 +533,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>LSD2026080800943352</t>
+          <t>LSD2026080100901233</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>185****6616</t>
+          <t>177****0229</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -590,27 +590,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>LSD2026080800943068</t>
+          <t>LSD2026080100898061</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>187****2309</t>
+          <t>158****7998</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -647,27 +647,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LSD2026080800942903</t>
+          <t>LSD2026080100895600</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>158****3037</t>
+          <t>135****5494</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -704,27 +704,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海复地活力城授权体验店</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LSD2026080800938677</t>
+          <t>LSD2026080100894959</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>152****6596</t>
+          <t>135****5494</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -761,27 +761,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海百联又一城授权体验店</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海百联又一城授权体验店</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>LSD2026080800937682</t>
+          <t>LSD2026080100901441</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>177****0313</t>
+          <t>186****9677</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -818,27 +818,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海美罗城授权体验店</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海美罗城授权体验店</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LSD2026080800937314</t>
+          <t>LSD2026080100899458</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>136****4038</t>
+          <t>177****3777</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -875,27 +875,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海长宁龙之梦授权体验店</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海长宁龙之梦授权体验店</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LSD2026080900951481</t>
+          <t>LSD2026080100896886</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>139****1145</t>
+          <t>177****3777</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -932,27 +932,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>上海爱飞</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LSD2026080900947256</t>
+          <t>LSD2026080100898888</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>153****8548</t>
+          <t>188****7855</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DJI上海中庚漫游城授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1004,12 +1004,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DJI上海中庚漫游城授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LSD2026080100898820</t>
+          <t>LSD2026080100898806</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>150****6552</t>
+          <t>188****7855</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LSD2026080100901233</t>
+          <t>LSD2026080100898731</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>177****0229</t>
+          <t>188****7855</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1103,12 +1103,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海百联又一城授权体验店</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1118,12 +1118,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海百联又一城授权体验店</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LSD2026080100898061</t>
+          <t>LSD2026080200903412</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>158****7998</t>
+          <t>137****9080</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1160,12 +1160,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海百联又一城授权体验店</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海百联又一城授权体验店</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LSD2026080100895600</t>
+          <t>LSD2026080300911904</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>135****5494</t>
+          <t>177****3777</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1217,12 +1217,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海长宁龙之梦授权体验店</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1232,12 +1232,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DJI上海复地活力城授权体验店</t>
+          <t>DJI上海长宁龙之梦授权体验店</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LSD2026080100894959</t>
+          <t>LSD2026080300911587</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>135****5494</t>
+          <t>138****4526</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1274,12 +1274,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DJI上海百联又一城授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1289,12 +1289,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DJI上海百联又一城授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LSD2026080100901441</t>
+          <t>LSD2026080400915298</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>186****9677</t>
+          <t>138****5533</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1331,7 +1331,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>LSD2026080100899458</t>
+          <t>LSD2026080400917951</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1388,12 +1388,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DJI上海长宁龙之梦授权体验店</t>
+          <t>DJI上海美罗城授权体验店</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1403,12 +1403,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DJI上海长宁龙之梦授权体验店</t>
+          <t>DJI上海美罗城授权体验店</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LSD2026080100896886</t>
+          <t>LSD2026080400917906</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1445,12 +1445,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1460,12 +1460,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LSD2026080100898888</t>
+          <t>LSD2026080500924466</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>188****7855</t>
+          <t>185****5918</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1502,12 +1502,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1517,12 +1517,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>LSD2026080100898806</t>
+          <t>LSD2026080500923088</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>188****7855</t>
+          <t>185****5918</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1559,12 +1559,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海天荟广场授权体验店</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1574,12 +1574,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海天荟广场授权体验店</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>LSD2026080100898731</t>
+          <t>LSD2026080500923845</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>188****7855</t>
+          <t>188****3772</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1616,12 +1616,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DJI上海百联又一城授权体验店</t>
+          <t>DJI上海漕河泾印象城授权体验店</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1631,12 +1631,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>DJI上海百联又一城授权体验店</t>
+          <t>DJI上海漕河泾印象城授权体验店</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LSD2026080200903412</t>
+          <t>LSD2026080500922902</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>137****9080</t>
+          <t>183****5937</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1673,12 +1673,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DJI上海百联又一城授权体验店</t>
+          <t>DJI上海长宁龙之梦授权体验店</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1688,12 +1688,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DJI上海百联又一城授权体验店</t>
+          <t>DJI上海长宁龙之梦授权体验店</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LSD2026080300911904</t>
+          <t>LSD2026080500923260</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1730,12 +1730,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DJI上海长宁龙之梦授权体验店</t>
+          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1745,12 +1745,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>DJI上海长宁龙之梦授权体验店</t>
+          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LSD2026080300911587</t>
+          <t>LSD2026080500922161</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>138****4526</t>
+          <t>189****1806</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1787,12 +1787,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海静安大融城授权体验店</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海静安大融城授权体验店</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>LSD2026080400915298</t>
+          <t>LSD2026080500923624</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1827,7 +1827,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>138****5533</t>
+          <t>139****1884</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1844,12 +1844,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DJI上海美罗城授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DJI上海美罗城授权体验店</t>
+          <t>DJI上海世博天地授权体验店</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>LSD2026080400917951</t>
+          <t>LSD2026080600925154</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>177****3777</t>
+          <t>189****6007</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1901,12 +1901,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DJI上海美罗城授权体验店</t>
+          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1916,12 +1916,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>DJI上海美罗城授权体验店</t>
+          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LSD2026080400917906</t>
+          <t>LSD2026080600925259</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>177****3777</t>
+          <t>167****1142</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1958,12 +1958,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海江桥万达授权体验店</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1973,12 +1973,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海江桥万达授权体验店</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>LSD2026080500924466</t>
+          <t>LSD2026080700936141</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>185****5918</t>
+          <t>186****8771</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2015,12 +2015,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海美罗城授权体验店</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海美罗城授权体验店</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>LSD2026080500923088</t>
+          <t>LSD2026080700935174</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>185****5918</t>
+          <t>130****8432</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2072,12 +2072,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DJI上海天荟广场授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2087,12 +2087,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>DJI上海天荟广场授权体验店</t>
+          <t>DJI上海长泰广场授权体验店</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>LSD2026080500923845</t>
+          <t>LSD2026080700931362</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>188****3772</t>
+          <t>186****7655</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2129,12 +2129,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DJI上海漕河泾印象城授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2144,12 +2144,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DJI上海漕河泾印象城授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LSD2026080500922902</t>
+          <t>LSD2026080800943589</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>183****5937</t>
+          <t>150****1153</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2186,12 +2186,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DJI上海长宁龙之梦授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2201,12 +2201,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>DJI上海长宁龙之梦授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>LSD2026080500923260</t>
+          <t>LSD2026080800943352</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>177****3777</t>
+          <t>185****6616</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2243,12 +2243,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2258,12 +2258,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>LSD2026080500922161</t>
+          <t>LSD2026080800943068</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>189****1806</t>
+          <t>187****2309</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2300,12 +2300,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DJI上海静安大融城授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2315,12 +2315,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>DJI上海静安大融城授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>LSD2026080500923624</t>
+          <t>LSD2026080800942903</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>139****1884</t>
+          <t>158****3037</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2357,12 +2357,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2372,12 +2372,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>DJI上海世博天地授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>LSD2026080600925154</t>
+          <t>LSD2026080800938677</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>189****6007</t>
+          <t>152****6596</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2414,12 +2414,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2429,12 +2429,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>LSD2026080600925259</t>
+          <t>LSD2026080800937682</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>167****1142</t>
+          <t>177****0313</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2471,12 +2471,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DJI上海江桥万达授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2486,12 +2486,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>DJI上海江桥万达授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>LSD2026080700936141</t>
+          <t>LSD2026080800937314</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>186****8771</t>
+          <t>136****4038</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2528,12 +2528,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DJI上海美罗城授权体验店</t>
+          <t>DJI上海天荟广场授权体验店</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2543,12 +2543,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>DJI上海美罗城授权体验店</t>
+          <t>DJI上海天荟广场授权体验店</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>LSD2026080700935174</t>
+          <t>LSD2026080800940954</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>130****8432</t>
+          <t>135****9693</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2585,12 +2585,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海江桥万达授权体验店</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2600,12 +2600,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>DJI上海长泰广场授权体验店</t>
+          <t>DJI上海江桥万达授权体验店</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>LSD2026080700931362</t>
+          <t>LSD2026080800939689</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>186****7655</t>
+          <t>150****0165</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DJI上海天荟广场授权体验店</t>
+          <t>DJI上海江桥万达授权体验店</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2657,12 +2657,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>DJI上海天荟广场授权体验店</t>
+          <t>DJI上海江桥万达授权体验店</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>LSD2026080800940954</t>
+          <t>LSD2026080800939622</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>135****9693</t>
+          <t>150****0165</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>LSD2026080800939689</t>
+          <t>LSD2026080800939401</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>DJI上海江桥万达授权体验店</t>
+          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2771,12 +2771,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>DJI上海江桥万达授权体验店</t>
+          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>LSD2026080800939622</t>
+          <t>LSD2026080800942684</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>150****0165</t>
+          <t>131****7661</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2813,12 +2813,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DJI上海江桥万达授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2828,12 +2828,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>DJI上海江桥万达授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>LSD2026080800939401</t>
+          <t>LSD2026080900951481</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>150****0165</t>
+          <t>139****1145</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2870,12 +2870,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2885,12 +2885,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>DJI上海陆家嘴中心L+mall授权体验店</t>
+          <t>DJI上海LCM置汇旭辉广场授权体验店</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>LSD2026080800942684</t>
+          <t>LSD2026080900947256</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>131****7661</t>
+          <t>153****8548</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">

</xml_diff>